<commit_message>
Log Session 8 Claude.md
</commit_message>
<xml_diff>
--- a/MasterSKU.xlsx
+++ b/MasterSKU.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hasil Minggu Ini\Essa-Store-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E7486E-0CCC-47AD-8C17-64665A66E8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29286872-8AB0-4913-B567-E709632D8021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
+    <workbookView xWindow="5025" yWindow="5025" windowWidth="28800" windowHeight="15345" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
   </bookViews>
   <sheets>
     <sheet name="Master SKU" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2394" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="643">
   <si>
     <t>Nomor SKU</t>
   </si>
@@ -1894,6 +1894,84 @@
   </si>
   <si>
     <t>ESSA Hijab Instan Olivia Size L Bergo Malay Oval Menutup Dada</t>
+  </si>
+  <si>
+    <t>PVR-INS-Noir</t>
+  </si>
+  <si>
+    <t>Pashmina Instan Kain Rayon Menutup Leher Dada</t>
+  </si>
+  <si>
+    <t>PVR-INS-Mahogany</t>
+  </si>
+  <si>
+    <t>PVR-INS-Ivory</t>
+  </si>
+  <si>
+    <t>PVR-INS-Navy</t>
+  </si>
+  <si>
+    <t>PVR-INS-Pink Blush</t>
+  </si>
+  <si>
+    <t>PVR-INS-Burgundy</t>
+  </si>
+  <si>
+    <t>PVR-INS-Cocoa</t>
+  </si>
+  <si>
+    <t>PVR-INS-Silver Mist</t>
+  </si>
+  <si>
+    <t>PVR-INS-Charcoal</t>
+  </si>
+  <si>
+    <t>PVR-INS-Mocha</t>
+  </si>
+  <si>
+    <t>PVR-INS-Taupe</t>
+  </si>
+  <si>
+    <t>PVR-INS-Sand</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Noir</t>
+  </si>
+  <si>
+    <t>Pashmina Polos Kain Rayon</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Mahogany</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Ivory</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Navy</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Pink Blush</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Burgundy</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Cocoa</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Silver Mist</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Charcoal</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Mocha</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Taupe</t>
+  </si>
+  <si>
+    <t>PVR-SWL-Sand</t>
   </si>
 </sst>
 </file>
@@ -1976,7 +2054,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1987,6 +2065,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8629,100 +8710,196 @@
       <c r="C598" s="1"/>
     </row>
     <row r="599" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A599" s="3"/>
-      <c r="B599" s="3"/>
+      <c r="A599" s="6" t="s">
+        <v>617</v>
+      </c>
+      <c r="B599" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="600" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A600" s="3"/>
-      <c r="B600" s="3"/>
+      <c r="A600" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="B600" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A601" s="3"/>
-      <c r="B601" s="3"/>
+      <c r="A601" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="B601" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="602" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A602" s="3"/>
-      <c r="B602" s="3"/>
+      <c r="A602" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="B602" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="603" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A603" s="3"/>
-      <c r="B603" s="3"/>
+      <c r="A603" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="B603" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="604" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A604" s="3"/>
-      <c r="B604" s="3"/>
+      <c r="A604" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="B604" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="605" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A605" s="3"/>
-      <c r="B605" s="3"/>
+      <c r="A605" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="B605" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="606" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A606" s="3"/>
-      <c r="B606" s="3"/>
+      <c r="A606" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="B606" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="607" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A607" s="3"/>
-      <c r="B607" s="3"/>
+      <c r="A607" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="B607" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="608" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A608" s="3"/>
-      <c r="B608" s="3"/>
+      <c r="A608" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="B608" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="609" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A609" s="3"/>
-      <c r="B609" s="3"/>
+      <c r="A609" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="B609" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="610" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A610" s="3"/>
-      <c r="B610" s="3"/>
+      <c r="A610" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="B610" s="6" t="s">
+        <v>618</v>
+      </c>
     </row>
     <row r="611" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A611" s="3"/>
-      <c r="B611" s="3"/>
+      <c r="A611" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="B611" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="612" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A612" s="3"/>
-      <c r="B612" s="3"/>
+      <c r="A612" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="B612" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="613" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A613" s="3"/>
-      <c r="B613" s="3"/>
+      <c r="A613" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="B613" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="614" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A614" s="3"/>
-      <c r="B614" s="3"/>
+      <c r="A614" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="B614" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="615" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A615" s="3"/>
-      <c r="B615" s="3"/>
+      <c r="A615" s="6" t="s">
+        <v>635</v>
+      </c>
+      <c r="B615" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="616" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A616" s="3"/>
-      <c r="B616" s="3"/>
+      <c r="A616" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="B616" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="617" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A617" s="3"/>
-      <c r="B617" s="3"/>
+      <c r="A617" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="B617" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="618" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A618" s="3"/>
-      <c r="B618" s="3"/>
+      <c r="A618" s="6" t="s">
+        <v>638</v>
+      </c>
+      <c r="B618" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="619" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A619" s="3"/>
-      <c r="B619" s="3"/>
+      <c r="A619" s="6" t="s">
+        <v>639</v>
+      </c>
+      <c r="B619" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="620" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A620" s="3"/>
-      <c r="B620" s="3"/>
+      <c r="A620" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="B620" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="621" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A621" s="3"/>
-      <c r="B621" s="3"/>
+      <c r="A621" s="6" t="s">
+        <v>641</v>
+      </c>
+      <c r="B621" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="622" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A622" s="3"/>
-      <c r="B622" s="3"/>
+      <c r="A622" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="B622" s="6" t="s">
+        <v>631</v>
+      </c>
     </row>
     <row r="623" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A623" s="3"/>

</xml_diff>

<commit_message>
Fix bug dropdown sku Penjahit pada Menu Payroll, Perubahan teknis untuk menu Invoice dan Profit Simulation
</commit_message>
<xml_diff>
--- a/MasterSKU.xlsx
+++ b/MasterSKU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hasil Minggu Ini\Essa-Store-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29286872-8AB0-4913-B567-E709632D8021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DEE776-7774-46D0-B023-E84675C88195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5025" yWindow="5025" windowWidth="28800" windowHeight="15345" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
+    <workbookView xWindow="2430" yWindow="3045" windowWidth="28800" windowHeight="15345" xr2:uid="{CECA2AD4-CD37-44C0-91AC-A97D1185B198}"/>
   </bookViews>
   <sheets>
     <sheet name="Master SKU" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2442" uniqueCount="643">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2610" uniqueCount="729">
   <si>
     <t>Nomor SKU</t>
   </si>
@@ -1972,6 +1972,264 @@
   </si>
   <si>
     <t>PVR-SWL-Sand</t>
+  </si>
+  <si>
+    <t>JSO-Almond (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Army (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Babypink (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Bata (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Beige (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Burgundy (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Caramel (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Choco (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Cokelat Tua (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Coksu (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Cream (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Dark Grey (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Denim (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Dusty Pink (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Fossil (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Grey (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Hazelnut (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Hitam (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Jotol (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Lilac (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Lime (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Maroon (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Mint (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Misty (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Moca (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Mustard (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Navy (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Olive (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Putih (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Putih Tulang (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Sage (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Smoke (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Softpink (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Taro (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Tosca (akrilik)</t>
+  </si>
+  <si>
+    <t>JSO-Turkish (akrilik)</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Noir</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Mahogany</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Ivory</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Navy</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Pink Blush</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Burgundy</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Cocoa</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Silver Mist</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Charcoal</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Mocha</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Taupe</t>
+  </si>
+  <si>
+    <t>BVR-TBN-Sand</t>
+  </si>
+  <si>
+    <t>Hijab Instan Bandana Tali Rayon</t>
+  </si>
+  <si>
+    <t>Hijab Instan Oval Putar</t>
+  </si>
+  <si>
+    <t>BJS-OP-Almond</t>
+  </si>
+  <si>
+    <t>BJS-OP-Army</t>
+  </si>
+  <si>
+    <t>BJS-OP-Bata</t>
+  </si>
+  <si>
+    <t>BJS-OP-Beige</t>
+  </si>
+  <si>
+    <t>BJS-OP-Burgundy</t>
+  </si>
+  <si>
+    <t>BJS-OP-Caramel</t>
+  </si>
+  <si>
+    <t>BJS-OP-Choco</t>
+  </si>
+  <si>
+    <t>BJS-OP-Cokelat Tua</t>
+  </si>
+  <si>
+    <t>BJS-OP-Coksu</t>
+  </si>
+  <si>
+    <t>BJS-OP-Cream</t>
+  </si>
+  <si>
+    <t>BJS-OP-Dark Grey</t>
+  </si>
+  <si>
+    <t>BJS-OP-Denim</t>
+  </si>
+  <si>
+    <t>BJS-OP-Dusty Pink</t>
+  </si>
+  <si>
+    <t>BJS-OP-Espresso</t>
+  </si>
+  <si>
+    <t>BJS-OP-Fossil</t>
+  </si>
+  <si>
+    <t>BJS-OP-Grey</t>
+  </si>
+  <si>
+    <t>BJS-OP-Hazelnut</t>
+  </si>
+  <si>
+    <t>BJS-OP-Hitam</t>
+  </si>
+  <si>
+    <t>BJS-OP-Jotol</t>
+  </si>
+  <si>
+    <t>BJS-OP-Latte</t>
+  </si>
+  <si>
+    <t>BJS-OP-Lilac</t>
+  </si>
+  <si>
+    <t>BJS-OP-Lime</t>
+  </si>
+  <si>
+    <t>BJS-OP-Maroon</t>
+  </si>
+  <si>
+    <t>BJS-OP-Mauve</t>
+  </si>
+  <si>
+    <t>BJS-OP-Moca</t>
+  </si>
+  <si>
+    <t>BJS-OP-Mustard</t>
+  </si>
+  <si>
+    <t>BJS-OP-Navy</t>
+  </si>
+  <si>
+    <t>BJS-OP-Olive</t>
+  </si>
+  <si>
+    <t>BJS-OP-Putih</t>
+  </si>
+  <si>
+    <t>BJS-OP-Putih Tulang</t>
+  </si>
+  <si>
+    <t>BJS-OP-Sage</t>
+  </si>
+  <si>
+    <t>BJS-OP-Smoke</t>
+  </si>
+  <si>
+    <t>BJS-OP-Softpink</t>
+  </si>
+  <si>
+    <t>BJS-OP-Taro</t>
+  </si>
+  <si>
+    <t>BJS-OP-Tosca</t>
+  </si>
+  <si>
+    <t>BJS-OP-Turkish</t>
   </si>
 </sst>
 </file>
@@ -2410,7 +2668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FD8F914-C444-47BA-9F60-B10F23023A52}">
-  <dimension ref="A1:C668"/>
+  <dimension ref="A1:C706"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" bestFit="1" customWidth="1"/>
@@ -8716,6 +8974,9 @@
       <c r="B599" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C599" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="600" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A600" s="6" t="s">
@@ -8724,6 +8985,9 @@
       <c r="B600" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C600" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A601" s="6" t="s">
@@ -8732,6 +8996,9 @@
       <c r="B601" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C601" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="602" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A602" s="6" t="s">
@@ -8740,6 +9007,9 @@
       <c r="B602" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C602" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="603" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A603" s="6" t="s">
@@ -8748,6 +9018,9 @@
       <c r="B603" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C603" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="604" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A604" s="6" t="s">
@@ -8756,6 +9029,9 @@
       <c r="B604" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C604" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="605" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A605" s="6" t="s">
@@ -8764,6 +9040,9 @@
       <c r="B605" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C605" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="606" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A606" s="6" t="s">
@@ -8772,6 +9051,9 @@
       <c r="B606" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C606" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="607" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A607" s="6" t="s">
@@ -8780,6 +9062,9 @@
       <c r="B607" s="6" t="s">
         <v>618</v>
       </c>
+      <c r="C607" s="2">
+        <v>23500</v>
+      </c>
     </row>
     <row r="608" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A608" s="6" t="s">
@@ -8788,302 +9073,1087 @@
       <c r="B608" s="6" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="609" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C608" s="2">
+        <v>23500</v>
+      </c>
+    </row>
+    <row r="609" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A609" s="6" t="s">
         <v>628</v>
       </c>
       <c r="B609" s="6" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="610" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C609" s="2">
+        <v>23500</v>
+      </c>
+    </row>
+    <row r="610" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A610" s="6" t="s">
         <v>629</v>
       </c>
       <c r="B610" s="6" t="s">
         <v>618</v>
       </c>
-    </row>
-    <row r="611" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C610" s="2">
+        <v>23500</v>
+      </c>
+    </row>
+    <row r="611" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A611" s="6" t="s">
         <v>630</v>
       </c>
       <c r="B611" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="612" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C611" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="612" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A612" s="6" t="s">
         <v>632</v>
       </c>
       <c r="B612" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="613" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C612" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="613" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A613" s="6" t="s">
         <v>633</v>
       </c>
       <c r="B613" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="614" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C613" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="614" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A614" s="6" t="s">
         <v>634</v>
       </c>
       <c r="B614" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="615" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C614" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="615" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A615" s="6" t="s">
         <v>635</v>
       </c>
       <c r="B615" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="616" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C615" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A616" s="6" t="s">
         <v>636</v>
       </c>
       <c r="B616" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="617" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C616" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A617" s="6" t="s">
         <v>637</v>
       </c>
       <c r="B617" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="618" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C617" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="618" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A618" s="6" t="s">
         <v>638</v>
       </c>
       <c r="B618" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="619" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C618" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="619" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A619" s="6" t="s">
         <v>639</v>
       </c>
       <c r="B619" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="620" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C619" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A620" s="6" t="s">
         <v>640</v>
       </c>
       <c r="B620" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="621" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C620" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A621" s="6" t="s">
         <v>641</v>
       </c>
       <c r="B621" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="622" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C621" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="622" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A622" s="6" t="s">
         <v>642</v>
       </c>
       <c r="B622" s="6" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="623" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A623" s="3"/>
-      <c r="B623" s="3"/>
-    </row>
-    <row r="624" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A624" s="3"/>
-      <c r="B624" s="3"/>
-    </row>
-    <row r="625" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A625" s="3"/>
-      <c r="B625" s="3"/>
-    </row>
-    <row r="626" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A626" s="3"/>
-      <c r="B626" s="3"/>
-    </row>
-    <row r="627" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A627" s="3"/>
-      <c r="B627" s="3"/>
-    </row>
-    <row r="628" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A628" s="3"/>
-      <c r="B628" s="3"/>
-    </row>
-    <row r="629" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A629" s="3"/>
-      <c r="B629" s="3"/>
-    </row>
-    <row r="630" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A630" s="3"/>
-      <c r="B630" s="3"/>
-    </row>
-    <row r="631" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A631" s="3"/>
-      <c r="B631" s="3"/>
-    </row>
-    <row r="632" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A632" s="3"/>
-      <c r="B632" s="3"/>
-    </row>
-    <row r="633" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A633" s="3"/>
-      <c r="B633" s="3"/>
-    </row>
-    <row r="634" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A634" s="3"/>
-      <c r="B634" s="3"/>
-    </row>
-    <row r="635" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A635" s="3"/>
-      <c r="B635" s="3"/>
-    </row>
-    <row r="636" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A636" s="3"/>
-      <c r="B636" s="3"/>
-    </row>
-    <row r="637" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A637" s="3"/>
-      <c r="B637" s="3"/>
-    </row>
-    <row r="638" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A638" s="3"/>
-      <c r="B638" s="3"/>
-    </row>
-    <row r="639" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A639" s="3"/>
-      <c r="B639" s="3"/>
-    </row>
-    <row r="640" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A640" s="3"/>
-      <c r="B640" s="3"/>
-    </row>
-    <row r="641" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A641" s="3"/>
-      <c r="B641" s="3"/>
-    </row>
-    <row r="642" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A642" s="3"/>
-      <c r="B642" s="3"/>
-    </row>
-    <row r="643" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A643" s="3"/>
-      <c r="B643" s="3"/>
-    </row>
-    <row r="644" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A644" s="3"/>
-      <c r="B644" s="3"/>
-    </row>
-    <row r="645" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A645" s="3"/>
-      <c r="B645" s="3"/>
-    </row>
-    <row r="646" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A646" s="3"/>
-      <c r="B646" s="3"/>
-    </row>
-    <row r="647" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A647" s="3"/>
-      <c r="B647" s="3"/>
-    </row>
-    <row r="648" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A648" s="3"/>
-      <c r="B648" s="3"/>
-    </row>
-    <row r="649" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A649" s="3"/>
-      <c r="B649" s="3"/>
-    </row>
-    <row r="650" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A650" s="3"/>
-      <c r="B650" s="3"/>
-    </row>
-    <row r="651" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A651" s="3"/>
-      <c r="B651" s="3"/>
-    </row>
-    <row r="652" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A652" s="3"/>
-      <c r="B652" s="3"/>
-    </row>
-    <row r="653" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A653" s="3"/>
-      <c r="B653" s="3"/>
-    </row>
-    <row r="654" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A654" s="3"/>
-      <c r="B654" s="3"/>
-    </row>
-    <row r="655" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A655" s="3"/>
-      <c r="B655" s="3"/>
-    </row>
-    <row r="656" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A656" s="3"/>
-      <c r="B656" s="3"/>
-    </row>
-    <row r="657" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A657" s="3"/>
-      <c r="B657" s="3"/>
-    </row>
-    <row r="658" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A658" s="3"/>
-      <c r="B658" s="3"/>
-    </row>
-    <row r="659" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A659" s="3"/>
-      <c r="B659" s="3"/>
-    </row>
-    <row r="660" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A660" s="3"/>
-      <c r="B660" s="3"/>
-    </row>
-    <row r="661" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A661" s="3"/>
-      <c r="B661" s="3"/>
-    </row>
-    <row r="662" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A662" s="3"/>
-      <c r="B662" s="3"/>
-    </row>
-    <row r="663" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A663" s="3"/>
-      <c r="B663" s="3"/>
-    </row>
-    <row r="664" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A664" s="3"/>
-      <c r="B664" s="3"/>
-    </row>
-    <row r="665" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A665" s="3"/>
-      <c r="B665" s="3"/>
-    </row>
-    <row r="666" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A666" s="3"/>
-      <c r="B666" s="3"/>
-    </row>
-    <row r="667" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A667" s="3"/>
-      <c r="B667" s="3"/>
-    </row>
-    <row r="668" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A668" s="3"/>
-      <c r="B668" s="3"/>
+      <c r="C622" s="2">
+        <v>23000</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A623" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="B623" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C623" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="624" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A624" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B624" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C624" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="625" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A625" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="B625" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C625" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="626" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A626" s="6" t="s">
+        <v>646</v>
+      </c>
+      <c r="B626" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C626" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="627" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A627" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="B627" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C627" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="628" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A628" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="B628" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C628" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="629" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A629" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="B629" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C629" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="630" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A630" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="B630" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C630" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="631" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A631" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="B631" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C631" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="632" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A632" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="B632" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C632" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="633" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A633" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="B633" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C633" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="634" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A634" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="B634" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C634" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="635" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A635" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="B635" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C635" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="636" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A636" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="B636" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C636" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="637" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A637" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="B637" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C637" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="638" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A638" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="B638" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C638" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="639" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A639" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="B639" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C639" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="640" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A640" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="B640" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C640" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="641" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A641" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="B641" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C641" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="642" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A642" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="B642" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C642" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="643" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A643" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="B643" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C643" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="644" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A644" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="B644" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C644" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="645" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A645" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="B645" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C645" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="646" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A646" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="B646" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C646" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="647" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A647" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="B647" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C647" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="648" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A648" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="B648" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C648" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="649" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A649" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="B649" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C649" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="650" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A650" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="B650" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C650" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="651" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A651" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="B651" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C651" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="652" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A652" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="B652" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C652" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="653" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A653" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="B653" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C653" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="654" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A654" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="B654" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C654" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="655" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A655" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="B655" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C655" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="656" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A656" s="6" t="s">
+        <v>676</v>
+      </c>
+      <c r="B656" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C656" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="657" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A657" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="B657" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C657" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="658" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A658" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="B658" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="C658" s="1">
+        <v>11700</v>
+      </c>
+    </row>
+    <row r="659" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A659" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="B659" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C659" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="660" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A660" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="B660" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C660" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="661" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A661" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="B661" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C661" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="662" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A662" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="B662" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C662" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="663" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A663" s="6" t="s">
+        <v>683</v>
+      </c>
+      <c r="B663" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C663" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="664" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A664" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="B664" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C664" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="665" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A665" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="B665" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C665" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="666" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A666" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="B666" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C666" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="667" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A667" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="B667" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C667" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="668" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A668" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="B668" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C668" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="669" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A669" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="B669" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C669" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="670" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A670" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="B670" s="3" t="s">
+        <v>691</v>
+      </c>
+      <c r="C670" s="2">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="671" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A671" s="3" t="s">
+        <v>693</v>
+      </c>
+      <c r="B671" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C671" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="672" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A672" s="3" t="s">
+        <v>694</v>
+      </c>
+      <c r="B672" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C672" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="673" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A673" s="3" t="s">
+        <v>695</v>
+      </c>
+      <c r="B673" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C673" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="674" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A674" s="3" t="s">
+        <v>696</v>
+      </c>
+      <c r="B674" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C674" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="675" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A675" s="3" t="s">
+        <v>697</v>
+      </c>
+      <c r="B675" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C675" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="676" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A676" s="3" t="s">
+        <v>698</v>
+      </c>
+      <c r="B676" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C676" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="677" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A677" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B677" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C677" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="678" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A678" s="3" t="s">
+        <v>700</v>
+      </c>
+      <c r="B678" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C678" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="679" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A679" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="B679" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C679" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="680" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A680" s="3" t="s">
+        <v>702</v>
+      </c>
+      <c r="B680" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C680" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="681" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A681" s="3" t="s">
+        <v>703</v>
+      </c>
+      <c r="B681" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C681" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="682" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A682" s="3" t="s">
+        <v>704</v>
+      </c>
+      <c r="B682" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C682" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="683" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A683" s="3" t="s">
+        <v>705</v>
+      </c>
+      <c r="B683" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C683" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="684" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A684" s="3" t="s">
+        <v>706</v>
+      </c>
+      <c r="B684" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C684" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="685" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A685" s="3" t="s">
+        <v>707</v>
+      </c>
+      <c r="B685" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C685" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="686" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A686" s="3" t="s">
+        <v>708</v>
+      </c>
+      <c r="B686" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C686" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="687" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A687" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="B687" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C687" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="688" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A688" s="3" t="s">
+        <v>710</v>
+      </c>
+      <c r="B688" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C688" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="689" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A689" s="3" t="s">
+        <v>711</v>
+      </c>
+      <c r="B689" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C689" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="690" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A690" s="3" t="s">
+        <v>712</v>
+      </c>
+      <c r="B690" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C690" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="691" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A691" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="B691" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C691" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="692" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A692" s="3" t="s">
+        <v>714</v>
+      </c>
+      <c r="B692" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C692" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="693" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A693" s="3" t="s">
+        <v>715</v>
+      </c>
+      <c r="B693" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C693" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="694" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A694" s="3" t="s">
+        <v>716</v>
+      </c>
+      <c r="B694" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C694" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="695" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A695" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="B695" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C695" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="696" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A696" s="3" t="s">
+        <v>718</v>
+      </c>
+      <c r="B696" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C696" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="697" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A697" s="3" t="s">
+        <v>719</v>
+      </c>
+      <c r="B697" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C697" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="698" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A698" s="3" t="s">
+        <v>720</v>
+      </c>
+      <c r="B698" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C698" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="699" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A699" s="3" t="s">
+        <v>721</v>
+      </c>
+      <c r="B699" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C699" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="700" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A700" s="3" t="s">
+        <v>722</v>
+      </c>
+      <c r="B700" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C700" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="701" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A701" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="B701" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C701" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="702" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A702" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="B702" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C702" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="703" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A703" s="3" t="s">
+        <v>725</v>
+      </c>
+      <c r="B703" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C703" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="704" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A704" s="3" t="s">
+        <v>726</v>
+      </c>
+      <c r="B704" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C704" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="705" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A705" s="3" t="s">
+        <v>727</v>
+      </c>
+      <c r="B705" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C705" s="2">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="706" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A706" s="3" t="s">
+        <v>728</v>
+      </c>
+      <c r="B706" s="1" t="s">
+        <v>692</v>
+      </c>
+      <c r="C706" s="2">
+        <v>12000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>